<commit_message>
Update after 0.3.0 publication
</commit_message>
<xml_diff>
--- a/terminology/CodeSystem-administrative-gender-cz.xlsx
+++ b/terminology/CodeSystem-administrative-gender-cz.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>4.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>

</xml_diff>